<commit_message>
feat: automate ClickHouse schema generation, mapping documentation, and DataHub excel upload preparation for PLM modules
</commit_message>
<xml_diff>
--- a/assets/upload_datahub_template.xlsx
+++ b/assets/upload_datahub_template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\E_Workspace\metadata-generator\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\E_Workspace\metadata-generator\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BC1AE7E1-E286-4284-8D5C-D7AD35CD9AB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3645C66-9C64-4D50-BF95-AEDEFDBC79CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="240" windowWidth="29040" windowHeight="15630" xr2:uid="{8E56EDC7-2087-40BF-BFDC-B0E1A816AF08}"/>
   </bookViews>
@@ -37,61 +37,133 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
-  <si>
-    <t>PROD</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>UAT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>STG</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Source</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="32">
   <si>
     <t>Column</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Column Desc</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>datahub_url</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>table_name</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>column_a</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>column_b</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>column_c</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>column_a_desc</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>column_b_desc</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>column_c_desc</t>
+    <t>PROD URN</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>STG URN</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Type</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>col_name</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>prev desc</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>sample row data</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>top unique values</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>other info</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>col_desc</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>confidence score</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>reasoning</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>score of col_desc by PM</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Score of confidence by PM</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Remark by PM</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Desc by PM</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Remarks by DevOps</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Evidence by DevOps</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Table</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{table_name}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{column_name_a}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{column_name_b}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{column_name_c}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{column_name_d}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{column_desc_a}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{column_desc_b}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{column_desc_c}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{column_desc_d}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TEST URN</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>desc</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>urn:li:dataset:(urn:li:dataPlatform:clickhouse,scmdp.plm.table_name,PROD)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -99,7 +171,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -114,6 +186,12 @@
       <family val="2"/>
       <charset val="136"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -138,8 +216,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -456,75 +537,162 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAD98EAC-6DBF-4FBF-8EBE-7E45648A12A2}">
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:T6"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.25" bestFit="1" customWidth="1"/>
+    <col min="1" max="3" width="11.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="22.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="24.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="D3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
+      <c r="E3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="D4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" t="s">
-        <v>7</v>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="D5" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" t="s">
-        <v>13</v>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="D6" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>